<commit_message>
cambio en usuario mike
</commit_message>
<xml_diff>
--- a/Llaves-servidor-ubuntu/Documentacion/Listado de usuarios.xlsx
+++ b/Llaves-servidor-ubuntu/Documentacion/Listado de usuarios.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="28">
   <si>
     <t xml:space="preserve">REGISTRO DE CREDENCIALES PARA USO DE VPN SERVER UBUNTU</t>
   </si>
@@ -28,16 +28,25 @@
     <t xml:space="preserve">Nombre completo</t>
   </si>
   <si>
+    <t xml:space="preserve">Sistema Operativo</t>
+  </si>
+  <si>
     <t xml:space="preserve">Nombre de usuario</t>
   </si>
   <si>
     <t xml:space="preserve">IP VPN Asignada</t>
   </si>
   <si>
-    <t xml:space="preserve">Private Key</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Public Key</t>
+    <t xml:space="preserve">Private Key-server</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public Key-server</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Private Key-windows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Public Key-Windows</t>
   </si>
   <si>
     <t xml:space="preserve">DNS</t>
@@ -46,12 +55,18 @@
     <t xml:space="preserve">Servidor Ubuntu</t>
   </si>
   <si>
+    <t xml:space="preserve">Linux</t>
+  </si>
+  <si>
     <t xml:space="preserve">1.1.1.1, 8.8.8.8</t>
   </si>
   <si>
     <t xml:space="preserve">Window Virtual 1</t>
   </si>
   <si>
+    <t xml:space="preserve">Windows</t>
+  </si>
+  <si>
     <t xml:space="preserve">Linux Fedora 1</t>
   </si>
   <si>
@@ -83,16 +98,23 @@
   </si>
   <si>
     <t xml:space="preserve">EIdDzkpyynBI0vUA+K3d4w46LG/2PiInaJjvzljAC20=</t>
+  </si>
+  <si>
+    <t xml:space="preserve">= okifike7ngr3infqflisl0g2ikml35dsef1garsvc00=</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vE6M/drp16y0SUk7RUsFZSulwr1nMuBmstwoGIgzFBU=</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="@"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -121,6 +143,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -171,32 +199,36 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -290,15 +322,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="B4:G23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <autoFilter ref="B4:G23"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabla1" displayName="Tabla1" ref="B4:J23" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <autoFilter ref="B4:J23"/>
+  <tableColumns count="9">
     <tableColumn id="1" name="Nombre completo"/>
-    <tableColumn id="2" name="Nombre de usuario"/>
-    <tableColumn id="3" name="IP VPN Asignada"/>
-    <tableColumn id="4" name="Private Key"/>
-    <tableColumn id="5" name="Public Key"/>
-    <tableColumn id="6" name="DNS"/>
+    <tableColumn id="2" name="Sistema Operativo"/>
+    <tableColumn id="3" name="Nombre de usuario"/>
+    <tableColumn id="4" name="IP VPN Asignada"/>
+    <tableColumn id="5" name="Private Key-server"/>
+    <tableColumn id="6" name="Public Key-server"/>
+    <tableColumn id="7" name="Private Key-windows"/>
+    <tableColumn id="8" name="Public Key-Windows"/>
+    <tableColumn id="9" name="DNS"/>
   </tableColumns>
 </table>
 </file>
@@ -480,53 +515,62 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:M23"/>
+  <dimension ref="B1:P23"/>
   <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="17.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="54.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="54.14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="19.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="54.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="54.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="42.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="49.15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18.57"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
       <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
       <c r="H2" s="3"/>
       <c r="I2" s="3"/>
       <c r="J2" s="3"/>
-      <c r="K2" s="3"/>
-      <c r="L2" s="3"/>
-      <c r="M2" s="3"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="5" t="s">
@@ -541,212 +585,278 @@
       <c r="G4" s="5" t="s">
         <v>6</v>
       </c>
+      <c r="H4" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="6"/>
+      <c r="B5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D5" s="6"/>
       <c r="E5" s="6"/>
       <c r="F5" s="6"/>
-      <c r="G5" s="6" t="s">
-        <v>8</v>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="6"/>
+      <c r="B6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
       <c r="F6" s="6"/>
-      <c r="G6" s="6" t="s">
-        <v>8</v>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C7" s="6"/>
+      <c r="B7" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
-      <c r="G7" s="6" t="s">
-        <v>8</v>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>12</v>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="D9" s="6" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>8</v>
+        <v>25</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C10" s="6"/>
       <c r="D10" s="6"/>
       <c r="E10" s="6"/>
       <c r="F10" s="6"/>
-      <c r="G10" s="6" t="s">
-        <v>8</v>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C11" s="6"/>
       <c r="D11" s="6"/>
       <c r="E11" s="6"/>
       <c r="F11" s="6"/>
-      <c r="G11" s="6" t="s">
-        <v>8</v>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C12" s="6"/>
       <c r="D12" s="6"/>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
-      <c r="G12" s="6" t="s">
-        <v>8</v>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C13" s="6"/>
       <c r="D13" s="6"/>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
-      <c r="G13" s="6" t="s">
-        <v>8</v>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C14" s="6"/>
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
-      <c r="G14" s="6" t="s">
-        <v>8</v>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="6"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
       <c r="F15" s="6"/>
-      <c r="G15" s="6" t="s">
-        <v>8</v>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C16" s="6"/>
       <c r="D16" s="6"/>
       <c r="E16" s="6"/>
       <c r="F16" s="6"/>
-      <c r="G16" s="6" t="s">
-        <v>8</v>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="6"/>
-      <c r="G17" s="6" t="s">
-        <v>8</v>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C18" s="6"/>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
-      <c r="G18" s="6" t="s">
-        <v>8</v>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
-      <c r="G19" s="6" t="s">
-        <v>8</v>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C20" s="6"/>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
-      <c r="G20" s="6" t="s">
-        <v>8</v>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C21" s="6"/>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
-      <c r="G21" s="6" t="s">
-        <v>8</v>
+      <c r="G21" s="6"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="6"/>
-      <c r="G22" s="6" t="s">
-        <v>8</v>
+      <c r="G22" s="6"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="6"/>
-      <c r="G23" s="6" t="s">
-        <v>8</v>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B1:G2"/>
+    <mergeCell ref="B1:J2"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>